<commit_message>
S127 3절: 마감 — 케이스 104/104 · pytest 1,665 · 미해결 58 → 58
회귀값 여덟 불변 · 감사 956·806·959·807 불변 · scan_ctrl 제어문자 0 · 탭 0.
갈래 넷 합 13분 10초 (①②③ 깨끗 · ④ 는 cdu-simul 과 겹쳐 오염).

미해결 이름 하나가 바뀌었다 — 「부가금이 실제로 서는 벌이 하나도 없다」 를
닫고 「초과가 나는 벌이 덱에만 있고 케이스 스터디 목록에는 없다」 를 올렸다.
②-39 는 판정까지다 — 상향 목표를 실으면 화면 어휘가 함께 움직인다.
그 몫은 값으로 쟀다: 4,000 → 5,294 kW 로 122,451,200원, 전액 부가금이다.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vr2pjktJG7fxenaYX4Ph5J
</commit_message>
<xml_diff>
--- a/output/casestudy_20260906.xlsx
+++ b/output/casestudy_20260906.xlsx
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>22.77347879996523</v>
+        <v>23.64374319999479</v>
       </c>
     </row>
     <row r="3">
@@ -596,7 +596,7 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>22.9550704001449</v>
+        <v>23.00087729981169</v>
       </c>
     </row>
     <row r="4">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>15.17589469999075</v>
+        <v>15.08662499999627</v>
       </c>
     </row>
     <row r="5">
@@ -700,7 +700,7 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>23.86988290003501</v>
+        <v>24.14168539992534</v>
       </c>
     </row>
     <row r="6">
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>25.62187600019388</v>
+        <v>25.61786060011946</v>
       </c>
     </row>
     <row r="7">
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>19.69503009994514</v>
+        <v>19.80059260013513</v>
       </c>
     </row>
     <row r="8">
@@ -856,7 +856,7 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>33.15327609982342</v>
+        <v>32.93654060014524</v>
       </c>
     </row>
   </sheetData>
@@ -9275,7 +9275,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>22.8 초</t>
+          <t>23.6 초</t>
         </is>
       </c>
     </row>
@@ -9299,7 +9299,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.2 초</t>
+          <t>15.1 초</t>
         </is>
       </c>
     </row>
@@ -9311,7 +9311,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>23.9 초</t>
+          <t>24.1 초</t>
         </is>
       </c>
     </row>
@@ -9335,7 +9335,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>19.7 초</t>
+          <t>19.8 초</t>
         </is>
       </c>
     </row>
@@ -9347,7 +9347,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>33.2 초</t>
+          <t>32.9 초</t>
         </is>
       </c>
     </row>
@@ -9359,7 +9359,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>169.0 초</t>
+          <t>170.2 초</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
S128 3절: 마감 - 케이스 118/118 · pytest 1,666 · 미해결 58 -> 58
회귀값 여덟 불변 · 감사 956·806·959·807 불변 · scan_ctrl 제어문자 0 · 탭 0.
갈래 넷 합 12분 51초 (넷 다 깨끗한 판).

미해결 이름 하나가 바뀌었다 - 「초과가 나는 벌이 덱에만 있고 케이스 스터디
목록에는 없다」 를 닫고 「덱 자료 주석이 용인 실측을 「케이스 스터디 목록에
없다」 고 적는다」 를 올렸다. 뒤엣것은 95세션 뒤로 서른세 판을 낡은 채
서 있던 주석 두 줄이고, 멈춤 규칙에 걸려 이름만 올린다.

pytest 분할 표에 127·128 두 열을 붙였다 - 127 값이 표에 없고 테스트 상태
칸에만 있었다. ② 가 16초 는 것은 케이스 벌이 하나 늘어서다. ③ 이 15초
줄었는데 시험은 58건 그대로다 - 까닭을 안 쟀다 (②-43 의 아홉 번째 판).

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vr2pjktJG7fxenaYX4Ph5J
</commit_message>
<xml_diff>
--- a/output/casestudy_20260906.xlsx
+++ b/output/casestudy_20260906.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>23.64374319999479</v>
+        <v>22.78387420019135</v>
       </c>
     </row>
     <row r="3">
@@ -596,7 +596,7 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>23.00087729981169</v>
+        <v>22.94120769994333</v>
       </c>
     </row>
     <row r="4">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>15.08662499999627</v>
+        <v>15.08017049985938</v>
       </c>
     </row>
     <row r="5">
@@ -700,7 +700,7 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>24.14168539992534</v>
+        <v>23.54686559992842</v>
       </c>
     </row>
     <row r="6">
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>25.61786060011946</v>
+        <v>25.51196929998696</v>
       </c>
     </row>
     <row r="7">
@@ -804,59 +804,111 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>19.80059260013513</v>
+        <v>19.7029236999806</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>C7 계약 부족형</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>general_b</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2023-04-25 ~ 2024-04-27</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>22284.79992</v>
+      </c>
+      <c r="E8" t="n">
+        <v>5293.44</v>
+      </c>
+      <c r="F8" t="n">
+        <v>5293</v>
+      </c>
+      <c r="G8" t="n">
+        <v>49.01480732181292</v>
+      </c>
+      <c r="H8" t="n">
+        <v>64.95604774948416</v>
+      </c>
+      <c r="I8" t="n">
+        <v>452804556.25</v>
+      </c>
+      <c r="J8" t="n">
+        <v>2898284725.008</v>
+      </c>
+      <c r="K8" t="n">
+        <v>3473540481.258</v>
+      </c>
+      <c r="L8" t="n">
+        <v>13.03582205801757</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>cache</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>24.07502040010877</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>R1 용인 실측</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>general_a_2</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>2025-08-28 ~ 2026-08-28</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="D9" t="n">
         <v>476.02327</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E9" t="n">
         <v>132.28</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F9" t="n">
         <v>132</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G9" t="n">
         <v>41.08229342532648</v>
       </c>
-      <c r="H8" t="n">
+      <c r="H9" t="n">
         <v>100.8144862191238</v>
       </c>
-      <c r="I8" t="n">
+      <c r="I9" t="n">
         <v>12422521.29032258</v>
       </c>
-      <c r="J8" t="n">
+      <c r="J9" t="n">
         <v>49597412.23</v>
       </c>
-      <c r="K8" t="n">
+      <c r="K9" t="n">
         <v>62019933.52032258</v>
       </c>
-      <c r="L8" t="n">
+      <c r="L9" t="n">
         <v>20.02988488572306</v>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>cache</t>
         </is>
       </c>
-      <c r="N8" t="n">
-        <v>32.93654060014524</v>
+      <c r="N9" t="n">
+        <v>33.19355620001443</v>
       </c>
     </row>
   </sheetData>
@@ -870,7 +922,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1700,7 +1752,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>R1 용인 실측</t>
+          <t>C7 계약 부족형</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1714,7 +1766,7 @@
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>132</v>
+        <v>5293</v>
       </c>
       <c r="G26" t="n">
         <v>0</v>
@@ -1736,28 +1788,28 @@
         <v>500</v>
       </c>
       <c r="C27" t="n">
-        <v>653924.9987308802</v>
+        <v>584346.8725203483</v>
       </c>
       <c r="D27" t="n">
-        <v>28.80135248983531</v>
+        <v>100</v>
       </c>
       <c r="E27" t="n">
-        <v>465585.7548272483</v>
+        <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>120</v>
+        <v>5204</v>
       </c>
       <c r="G27" t="n">
-        <v>1371755.161290321</v>
+        <v>12693662.5</v>
       </c>
       <c r="H27" t="n">
-        <v>21832794.0374309</v>
+        <v>78883246.71788597</v>
       </c>
       <c r="I27" t="n">
-        <v>23204549.19872123</v>
+        <v>109749224.7603021</v>
       </c>
       <c r="J27" t="n">
-        <v>23204549.19872123</v>
+        <v>109749224.7603021</v>
       </c>
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr"/>
@@ -1767,28 +1819,28 @@
         <v>1000</v>
       </c>
       <c r="C28" t="n">
-        <v>1307849.99746176</v>
+        <v>1168693.745040697</v>
       </c>
       <c r="D28" t="n">
-        <v>15.68075433387349</v>
+        <v>100</v>
       </c>
       <c r="E28" t="n">
-        <v>1102769.252304211</v>
+        <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>120</v>
+        <v>5198</v>
       </c>
       <c r="G28" t="n">
-        <v>1421135.161290321</v>
+        <v>17911015</v>
       </c>
       <c r="H28" t="n">
-        <v>23715557.01062761</v>
+        <v>157766493.4357724</v>
       </c>
       <c r="I28" t="n">
-        <v>25136692.17191793</v>
+        <v>214786217.6287827</v>
       </c>
       <c r="J28" t="n">
-        <v>25136692.17191793</v>
+        <v>214786217.6287827</v>
       </c>
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr"/>
@@ -1798,39 +1850,167 @@
         <v>2000</v>
       </c>
       <c r="C29" t="n">
-        <v>2615699.994923521</v>
+        <v>2337387.490081393</v>
       </c>
       <c r="D29" t="n">
-        <v>8.179882063646165</v>
+        <v>100</v>
       </c>
       <c r="E29" t="n">
-        <v>2401738.820199978</v>
+        <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>120</v>
+        <v>5186</v>
       </c>
       <c r="G29" t="n">
-        <v>1421135.161290321</v>
+        <v>21835085</v>
       </c>
       <c r="H29" t="n">
-        <v>24660958.77724204</v>
+        <v>315532986.8715444</v>
       </c>
       <c r="I29" t="n">
-        <v>26082093.93853237</v>
+        <v>381629820.0461593</v>
       </c>
       <c r="J29" t="n">
-        <v>26082093.93853237</v>
+        <v>381629820.0461593</v>
       </c>
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr"/>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>R1 용인 실측</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="n">
+        <v>132</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="B31" t="n">
+        <v>500</v>
+      </c>
+      <c r="C31" t="n">
+        <v>653924.9987308802</v>
+      </c>
+      <c r="D31" t="n">
+        <v>28.80135248983531</v>
+      </c>
+      <c r="E31" t="n">
+        <v>465585.7548272483</v>
+      </c>
+      <c r="F31" t="n">
+        <v>120</v>
+      </c>
+      <c r="G31" t="n">
+        <v>1371755.161290321</v>
+      </c>
+      <c r="H31" t="n">
+        <v>21832794.0374309</v>
+      </c>
+      <c r="I31" t="n">
+        <v>23204549.19872123</v>
+      </c>
+      <c r="J31" t="n">
+        <v>23204549.19872123</v>
+      </c>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="B32" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C32" t="n">
+        <v>1307849.99746176</v>
+      </c>
+      <c r="D32" t="n">
+        <v>15.68075433387349</v>
+      </c>
+      <c r="E32" t="n">
+        <v>1102769.252304211</v>
+      </c>
+      <c r="F32" t="n">
+        <v>120</v>
+      </c>
+      <c r="G32" t="n">
+        <v>1421135.161290321</v>
+      </c>
+      <c r="H32" t="n">
+        <v>23715557.01062761</v>
+      </c>
+      <c r="I32" t="n">
+        <v>25136692.17191793</v>
+      </c>
+      <c r="J32" t="n">
+        <v>25136692.17191793</v>
+      </c>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="B33" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C33" t="n">
+        <v>2615699.994923521</v>
+      </c>
+      <c r="D33" t="n">
+        <v>8.179882063646165</v>
+      </c>
+      <c r="E33" t="n">
+        <v>2401738.820199978</v>
+      </c>
+      <c r="F33" t="n">
+        <v>120</v>
+      </c>
+      <c r="G33" t="n">
+        <v>1421135.161290321</v>
+      </c>
+      <c r="H33" t="n">
+        <v>24660958.77724204</v>
+      </c>
+      <c r="I33" t="n">
+        <v>26082093.93853237</v>
+      </c>
+      <c r="J33" t="n">
+        <v>26082093.93853237</v>
+      </c>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
+    </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
     <mergeCell ref="A18:A21"/>
     <mergeCell ref="A26:A29"/>
     <mergeCell ref="A2:A5"/>
     <mergeCell ref="A6:A9"/>
     <mergeCell ref="A14:A17"/>
+    <mergeCell ref="A30:A33"/>
     <mergeCell ref="A10:A13"/>
     <mergeCell ref="A22:A25"/>
   </mergeCells>
@@ -1844,7 +2024,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I148"/>
+  <dimension ref="A1:I169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5491,7 +5671,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>R1 용인 실측</t>
+          <t>C7 계약 부족형</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -5503,13 +5683,13 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>1371755.161290321</v>
+        <v>-54359243.75</v>
       </c>
       <c r="E128" t="n">
-        <v>1019989.032258064</v>
+        <v>-56468883.75</v>
       </c>
       <c r="F128" t="n">
-        <v>1421135.161290321</v>
+        <v>-54359243.75</v>
       </c>
       <c r="G128" t="inlineStr">
         <is>
@@ -5518,11 +5698,11 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>평탄형</t>
+          <t>기준</t>
         </is>
       </c>
       <c r="I128" t="n">
-        <v>28.22716233887541</v>
+        <v>3.735933597235309</v>
       </c>
     </row>
     <row r="129">
@@ -5532,13 +5712,13 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>21832794.0374309</v>
+        <v>198235738.4790244</v>
       </c>
       <c r="E129" t="n">
-        <v>19707849.27224809</v>
+        <v>197954047.4566307</v>
       </c>
       <c r="F129" t="n">
-        <v>23383003.92461409</v>
+        <v>198235738.4790244</v>
       </c>
       <c r="G129" t="inlineStr">
         <is>
@@ -5547,11 +5727,11 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>평탄형</t>
+          <t>기준</t>
         </is>
       </c>
       <c r="I129" t="n">
-        <v>15.71720495884344</v>
+        <v>0.1420990102768526</v>
       </c>
     </row>
     <row r="130">
@@ -5561,13 +5741,13 @@
         </is>
       </c>
       <c r="D130" t="n">
-        <v>22552939.7162026</v>
+        <v>145590002.7194409</v>
       </c>
       <c r="E130" t="n">
-        <v>20181372.38521974</v>
+        <v>141091876.8111548</v>
       </c>
       <c r="F130" t="n">
-        <v>24100050.37364634</v>
+        <v>146601251.3777847</v>
       </c>
       <c r="G130" t="inlineStr">
         <is>
@@ -5580,7 +5760,7 @@
         </is>
       </c>
       <c r="I130" t="n">
-        <v>16.26004065415448</v>
+        <v>3.758067898364988</v>
       </c>
     </row>
     <row r="131">
@@ -5590,13 +5770,13 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>22552939.7162026</v>
+        <v>145590002.7194409</v>
       </c>
       <c r="E131" t="n">
-        <v>20181372.38521974</v>
+        <v>141091876.8111548</v>
       </c>
       <c r="F131" t="n">
-        <v>24100050.37364634</v>
+        <v>146601251.3777847</v>
       </c>
       <c r="G131" t="inlineStr">
         <is>
@@ -5609,7 +5789,7 @@
         </is>
       </c>
       <c r="I131" t="n">
-        <v>16.26004065415447</v>
+        <v>3.758067898364988</v>
       </c>
     </row>
     <row r="132">
@@ -5619,13 +5799,13 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>120</v>
+        <v>5204</v>
       </c>
       <c r="E132" t="n">
-        <v>120</v>
+        <v>5201</v>
       </c>
       <c r="F132" t="n">
-        <v>122</v>
+        <v>5209</v>
       </c>
       <c r="G132" t="inlineStr">
         <is>
@@ -5638,7 +5818,7 @@
         </is>
       </c>
       <c r="I132" t="n">
-        <v>1.639344262295082</v>
+        <v>0.1535803417162603</v>
       </c>
     </row>
     <row r="133">
@@ -5648,26 +5828,26 @@
         </is>
       </c>
       <c r="D133" t="n">
-        <v>653924.9987308802</v>
+        <v>584346.8725203483</v>
       </c>
       <c r="E133" t="n">
-        <v>653917.3979531642</v>
+        <v>584298.3051197322</v>
       </c>
       <c r="F133" t="n">
-        <v>653931.4335780952</v>
+        <v>584399.679278902</v>
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>첨예형</t>
+          <t>평탄형</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>평탄형</t>
+          <t>첨예형</t>
         </is>
       </c>
       <c r="I133" t="n">
-        <v>0.002146345046327881</v>
+        <v>0.01734671711232556</v>
       </c>
     </row>
     <row r="134">
@@ -5701,13 +5881,13 @@
         </is>
       </c>
       <c r="D135" t="n">
-        <v>2838081.612903226</v>
+        <v>-48347003.75</v>
       </c>
       <c r="E135" t="n">
-        <v>2488601.935483871</v>
+        <v>-52474763.75</v>
       </c>
       <c r="F135" t="n">
-        <v>2838081.612903226</v>
+        <v>-46220203.75</v>
       </c>
       <c r="G135" t="inlineStr">
         <is>
@@ -5720,7 +5900,7 @@
         </is>
       </c>
       <c r="I135" t="n">
-        <v>12.31394036839743</v>
+        <v>11.91917705394148</v>
       </c>
     </row>
     <row r="136">
@@ -5730,13 +5910,13 @@
         </is>
       </c>
       <c r="D136" t="n">
-        <v>22279561.62896263</v>
+        <v>273905077.3980494</v>
       </c>
       <c r="E136" t="n">
-        <v>19622065.81315529</v>
+        <v>273341695.35326</v>
       </c>
       <c r="F136" t="n">
-        <v>23884897.59634926</v>
+        <v>273905077.3980494</v>
       </c>
       <c r="G136" t="inlineStr">
         <is>
@@ -5745,11 +5925,11 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>평탄형</t>
+          <t>기준</t>
         </is>
       </c>
       <c r="I136" t="n">
-        <v>17.84739401120788</v>
+        <v>0.2056851410500091</v>
       </c>
     </row>
     <row r="137">
@@ -5759,13 +5939,13 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>24504239.10251102</v>
+        <v>250781074.8714399</v>
       </c>
       <c r="E137" t="n">
-        <v>21550431.56860603</v>
+        <v>232274390.6218596</v>
       </c>
       <c r="F137" t="n">
-        <v>26109575.06989764</v>
+        <v>255332003.846559</v>
       </c>
       <c r="G137" t="inlineStr">
         <is>
@@ -5778,7 +5958,7 @@
         </is>
       </c>
       <c r="I137" t="n">
-        <v>17.46157679351877</v>
+        <v>9.03044384461726</v>
       </c>
     </row>
     <row r="138">
@@ -5788,13 +5968,13 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>24504239.10251102</v>
+        <v>250781074.8714399</v>
       </c>
       <c r="E138" t="n">
-        <v>21550431.56860603</v>
+        <v>232274390.6218596</v>
       </c>
       <c r="F138" t="n">
-        <v>26109575.06989764</v>
+        <v>255332003.846559</v>
       </c>
       <c r="G138" t="inlineStr">
         <is>
@@ -5807,7 +5987,7 @@
         </is>
       </c>
       <c r="I138" t="n">
-        <v>17.46157679351876</v>
+        <v>9.03044384461726</v>
       </c>
     </row>
     <row r="139">
@@ -5817,13 +5997,13 @@
         </is>
       </c>
       <c r="D139" t="n">
-        <v>120</v>
+        <v>5198</v>
       </c>
       <c r="E139" t="n">
-        <v>120</v>
+        <v>5192</v>
       </c>
       <c r="F139" t="n">
-        <v>122</v>
+        <v>5207</v>
       </c>
       <c r="G139" t="inlineStr">
         <is>
@@ -5836,7 +6016,7 @@
         </is>
       </c>
       <c r="I139" t="n">
-        <v>1.639344262295082</v>
+        <v>0.2880737468792011</v>
       </c>
     </row>
     <row r="140">
@@ -5846,26 +6026,26 @@
         </is>
       </c>
       <c r="D140" t="n">
-        <v>1307849.99746176</v>
+        <v>1168693.745040697</v>
       </c>
       <c r="E140" t="n">
-        <v>1307834.795906328</v>
+        <v>1168596.610239464</v>
       </c>
       <c r="F140" t="n">
-        <v>1307862.86715619</v>
+        <v>1168799.358557804</v>
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>첨예형</t>
+          <t>평탄형</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>평탄형</t>
+          <t>첨예형</t>
         </is>
       </c>
       <c r="I140" t="n">
-        <v>0.002146345046327881</v>
+        <v>0.01734671711232556</v>
       </c>
     </row>
     <row r="141">
@@ -5899,13 +6079,13 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>2838081.612903226</v>
+        <v>-43825083.75</v>
       </c>
       <c r="E142" t="n">
-        <v>2488601.935483871</v>
+        <v>-50617843.75</v>
       </c>
       <c r="F142" t="n">
-        <v>2838081.612903226</v>
+        <v>-39506483.75</v>
       </c>
       <c r="G142" t="inlineStr">
         <is>
@@ -5918,7 +6098,7 @@
         </is>
       </c>
       <c r="I142" t="n">
-        <v>12.31394036839743</v>
+        <v>21.95146844831769</v>
       </c>
     </row>
     <row r="143">
@@ -5928,13 +6108,13 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>23272029.67227682</v>
+        <v>425243755.2360973</v>
       </c>
       <c r="E143" t="n">
-        <v>20452277.86005339</v>
+        <v>424105698.3038983</v>
       </c>
       <c r="F143" t="n">
-        <v>24555709.08009543</v>
+        <v>425243755.2360973</v>
       </c>
       <c r="G143" t="inlineStr">
         <is>
@@ -5943,11 +6123,11 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>평탄형</t>
+          <t>기준</t>
         </is>
       </c>
       <c r="I143" t="n">
-        <v>16.71070139598712</v>
+        <v>0.2676246078127936</v>
       </c>
     </row>
     <row r="144">
@@ -5957,13 +6137,13 @@
         </is>
       </c>
       <c r="D144" t="n">
-        <v>25496707.14582521</v>
+        <v>411147406.6891804</v>
       </c>
       <c r="E144" t="n">
-        <v>22331217.54167268</v>
+        <v>386414083.0198159</v>
       </c>
       <c r="F144" t="n">
-        <v>26780386.55364382</v>
+        <v>419828404.5632014</v>
       </c>
       <c r="G144" t="inlineStr">
         <is>
@@ -5976,7 +6156,7 @@
         </is>
       </c>
       <c r="I144" t="n">
-        <v>16.61353544340745</v>
+        <v>7.95904259459302</v>
       </c>
     </row>
     <row r="145">
@@ -5986,13 +6166,13 @@
         </is>
       </c>
       <c r="D145" t="n">
-        <v>25496707.14582521</v>
+        <v>411147406.6891804</v>
       </c>
       <c r="E145" t="n">
-        <v>22331217.54167268</v>
+        <v>386414083.0198159</v>
       </c>
       <c r="F145" t="n">
-        <v>26780386.55364381</v>
+        <v>419828404.5632014</v>
       </c>
       <c r="G145" t="inlineStr">
         <is>
@@ -6005,7 +6185,7 @@
         </is>
       </c>
       <c r="I145" t="n">
-        <v>16.61353544340744</v>
+        <v>7.95904259459302</v>
       </c>
     </row>
     <row r="146">
@@ -6015,13 +6195,13 @@
         </is>
       </c>
       <c r="D146" t="n">
-        <v>120</v>
+        <v>5186</v>
       </c>
       <c r="E146" t="n">
-        <v>120</v>
+        <v>5175</v>
       </c>
       <c r="F146" t="n">
-        <v>122</v>
+        <v>5204</v>
       </c>
       <c r="G146" t="inlineStr">
         <is>
@@ -6034,7 +6214,7 @@
         </is>
       </c>
       <c r="I146" t="n">
-        <v>1.639344262295082</v>
+        <v>0.5572636433512683</v>
       </c>
     </row>
     <row r="147">
@@ -6044,26 +6224,26 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>2615699.994923521</v>
+        <v>2337387.490081393</v>
       </c>
       <c r="E147" t="n">
-        <v>2615669.591812657</v>
+        <v>2337193.220478929</v>
       </c>
       <c r="F147" t="n">
-        <v>2615725.734312381</v>
+        <v>2337598.717115608</v>
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>첨예형</t>
+          <t>평탄형</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>평탄형</t>
+          <t>첨예형</t>
         </is>
       </c>
       <c r="I147" t="n">
-        <v>0.002146345046327881</v>
+        <v>0.01734671711232556</v>
       </c>
     </row>
     <row r="148">
@@ -6087,8 +6267,607 @@
       </c>
       <c r="I148" t="inlineStr"/>
     </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>R1 용인 실측</t>
+        </is>
+      </c>
+      <c r="B149" t="n">
+        <v>500</v>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>기본요금 절감액(원)</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>1371755.161290321</v>
+      </c>
+      <c r="E149" t="n">
+        <v>1019989.032258064</v>
+      </c>
+      <c r="F149" t="n">
+        <v>1421135.161290321</v>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="I149" t="n">
+        <v>28.22716233887541</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>전력량요금 절감액(원)</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>21832794.0374309</v>
+      </c>
+      <c r="E150" t="n">
+        <v>19707849.27224809</v>
+      </c>
+      <c r="F150" t="n">
+        <v>23383003.92461409</v>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="I150" t="n">
+        <v>15.71720495884344</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>절감액(원)</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>22552939.7162026</v>
+      </c>
+      <c r="E151" t="n">
+        <v>20181372.38521974</v>
+      </c>
+      <c r="F151" t="n">
+        <v>24100050.37364634</v>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="I151" t="n">
+        <v>16.26004065415448</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>12개월 환산 절감액(원)</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>22552939.7162026</v>
+      </c>
+      <c r="E152" t="n">
+        <v>20181372.38521974</v>
+      </c>
+      <c r="F152" t="n">
+        <v>24100050.37364634</v>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="I152" t="n">
+        <v>16.26004065415447</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>요금적용전력(kW)</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>120</v>
+      </c>
+      <c r="E153" t="n">
+        <v>120</v>
+      </c>
+      <c r="F153" t="n">
+        <v>122</v>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="I153" t="n">
+        <v>1.639344262295082</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>발전량(kWh)</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>653924.9987308802</v>
+      </c>
+      <c r="E154" t="n">
+        <v>653917.3979531642</v>
+      </c>
+      <c r="F154" t="n">
+        <v>653931.4335780952</v>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="I154" t="n">
+        <v>0.002146345046327881</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>회수기간(년)</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr"/>
+      <c r="E155" t="inlineStr"/>
+      <c r="F155" t="inlineStr"/>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="B156" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>기본요금 절감액(원)</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>2838081.612903226</v>
+      </c>
+      <c r="E156" t="n">
+        <v>2488601.935483871</v>
+      </c>
+      <c r="F156" t="n">
+        <v>2838081.612903226</v>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="I156" t="n">
+        <v>12.31394036839743</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>전력량요금 절감액(원)</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>22279561.62896263</v>
+      </c>
+      <c r="E157" t="n">
+        <v>19622065.81315529</v>
+      </c>
+      <c r="F157" t="n">
+        <v>23884897.59634926</v>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="I157" t="n">
+        <v>17.84739401120788</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>절감액(원)</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>24504239.10251102</v>
+      </c>
+      <c r="E158" t="n">
+        <v>21550431.56860603</v>
+      </c>
+      <c r="F158" t="n">
+        <v>26109575.06989764</v>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="I158" t="n">
+        <v>17.46157679351877</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>12개월 환산 절감액(원)</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>24504239.10251102</v>
+      </c>
+      <c r="E159" t="n">
+        <v>21550431.56860603</v>
+      </c>
+      <c r="F159" t="n">
+        <v>26109575.06989764</v>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="I159" t="n">
+        <v>17.46157679351876</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>요금적용전력(kW)</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>120</v>
+      </c>
+      <c r="E160" t="n">
+        <v>120</v>
+      </c>
+      <c r="F160" t="n">
+        <v>122</v>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="I160" t="n">
+        <v>1.639344262295082</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>발전량(kWh)</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>1307849.99746176</v>
+      </c>
+      <c r="E161" t="n">
+        <v>1307834.795906328</v>
+      </c>
+      <c r="F161" t="n">
+        <v>1307862.86715619</v>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="I161" t="n">
+        <v>0.002146345046327881</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>회수기간(년)</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr"/>
+      <c r="E162" t="inlineStr"/>
+      <c r="F162" t="inlineStr"/>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="B163" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>기본요금 절감액(원)</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>2838081.612903226</v>
+      </c>
+      <c r="E163" t="n">
+        <v>2488601.935483871</v>
+      </c>
+      <c r="F163" t="n">
+        <v>2838081.612903226</v>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="I163" t="n">
+        <v>12.31394036839743</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>전력량요금 절감액(원)</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>23272029.67227682</v>
+      </c>
+      <c r="E164" t="n">
+        <v>20452277.86005339</v>
+      </c>
+      <c r="F164" t="n">
+        <v>24555709.08009543</v>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="I164" t="n">
+        <v>16.71070139598712</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>절감액(원)</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>25496707.14582521</v>
+      </c>
+      <c r="E165" t="n">
+        <v>22331217.54167268</v>
+      </c>
+      <c r="F165" t="n">
+        <v>26780386.55364382</v>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="I165" t="n">
+        <v>16.61353544340745</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>12개월 환산 절감액(원)</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>25496707.14582521</v>
+      </c>
+      <c r="E166" t="n">
+        <v>22331217.54167268</v>
+      </c>
+      <c r="F166" t="n">
+        <v>26780386.55364381</v>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="I166" t="n">
+        <v>16.61353544340744</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>요금적용전력(kW)</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>120</v>
+      </c>
+      <c r="E167" t="n">
+        <v>120</v>
+      </c>
+      <c r="F167" t="n">
+        <v>122</v>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="I167" t="n">
+        <v>1.639344262295082</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>발전량(kWh)</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>2615699.994923521</v>
+      </c>
+      <c r="E168" t="n">
+        <v>2615669.591812657</v>
+      </c>
+      <c r="F168" t="n">
+        <v>2615725.734312381</v>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="I168" t="n">
+        <v>0.002146345046327881</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>회수기간(년)</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr"/>
+      <c r="E169" t="inlineStr"/>
+      <c r="F169" t="inlineStr"/>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr"/>
+    </row>
   </sheetData>
-  <mergeCells count="28">
+  <mergeCells count="32">
     <mergeCell ref="A44:A64"/>
     <mergeCell ref="B86:B92"/>
     <mergeCell ref="B44:B50"/>
@@ -6106,13 +6885,17 @@
     <mergeCell ref="B30:B36"/>
     <mergeCell ref="B114:B120"/>
     <mergeCell ref="B79:B85"/>
+    <mergeCell ref="B163:B169"/>
     <mergeCell ref="B51:B57"/>
     <mergeCell ref="B135:B141"/>
     <mergeCell ref="A65:A85"/>
+    <mergeCell ref="A149:A169"/>
     <mergeCell ref="A86:A106"/>
     <mergeCell ref="B72:B78"/>
     <mergeCell ref="A2:A22"/>
     <mergeCell ref="B100:B106"/>
+    <mergeCell ref="B149:B155"/>
+    <mergeCell ref="B156:B162"/>
     <mergeCell ref="B121:B127"/>
     <mergeCell ref="B2:B8"/>
     <mergeCell ref="B93:B99"/>
@@ -6128,7 +6911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6479,7 +7262,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>R1 용인 실측</t>
+          <t>C7 계약 부족형</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -6488,13 +7271,13 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>62942872.33519353</v>
+        <v>3473540481.258</v>
       </c>
       <c r="D20" t="n">
-        <v>-922938.8148709536</v>
+        <v>0</v>
       </c>
       <c r="E20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -6504,13 +7287,13 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>62019933.52032258</v>
+        <v>3438616925.448</v>
       </c>
       <c r="D21" t="n">
-        <v>0</v>
+        <v>34923555.81000042</v>
       </c>
       <c r="E21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -6520,38 +7303,92 @@
         </is>
       </c>
       <c r="C22" t="n">
+        <v>3491538784.641</v>
+      </c>
+      <c r="D22" t="n">
+        <v>-17998303.3829999</v>
+      </c>
+      <c r="E22" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>R1 용인 실측</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>62942872.33519353</v>
+      </c>
+      <c r="D23" t="n">
+        <v>-922938.8148709536</v>
+      </c>
+      <c r="E23" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>62019933.52032258</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
         <v>68875492.43619356</v>
       </c>
-      <c r="D22" t="n">
+      <c r="D25" t="n">
         <v>-6855558.915870979</v>
       </c>
-      <c r="E22" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" t="inlineStr">
+      <c r="E25" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" t="inlineStr">
         <is>
           <t>IV</t>
         </is>
       </c>
-      <c r="C23" t="n">
+      <c r="C26" t="n">
         <v>68298776.96832258</v>
       </c>
-      <c r="D23" t="n">
+      <c r="D26" t="n">
         <v>-6278843.447999999</v>
       </c>
-      <c r="E23" t="b">
+      <c r="E26" t="b">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
     <mergeCell ref="A8:A10"/>
+    <mergeCell ref="A23:A26"/>
     <mergeCell ref="A2:A4"/>
     <mergeCell ref="A17:A19"/>
+    <mergeCell ref="A20:A22"/>
     <mergeCell ref="A11:A13"/>
-    <mergeCell ref="A20:A23"/>
     <mergeCell ref="A5:A7"/>
     <mergeCell ref="A14:A16"/>
   </mergeCells>
@@ -6565,7 +7402,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7271,7 +8108,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>R1 용인 실측</t>
+          <t>C7 계약 부족형</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -7280,10 +8117,10 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>0</v>
+        <v>34923555.81000042</v>
       </c>
       <c r="D32" t="n">
-        <v>0</v>
+        <v>34923555.81000042</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -7292,7 +8129,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>II → II</t>
+          <t>I → II</t>
         </is>
       </c>
     </row>
@@ -7313,7 +8150,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>계약 290 kW (실제 값)</t>
+          <t>계약 4,000 kW (합성 조건)</t>
         </is>
       </c>
     </row>
@@ -7324,10 +8161,10 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>124225.2129032239</v>
+        <v>4528045.5625</v>
       </c>
       <c r="D34" t="n">
-        <v>124225.2129032239</v>
+        <v>4528045.5625</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -7346,7 +8183,9 @@
           <t>7.6 ESS</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
+      <c r="C35" t="n">
+        <v>25544657.48527241</v>
+      </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
@@ -7355,7 +8194,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>최소 규격 미달 — 필요 출력 25.3 kW &lt; 상업용 최소 50 kW</t>
+          <t>목표 5,180 kW (기준 5,293.0 → 실제 5,180.0) · 150 kW / 100 kWh · 회수 10.3년</t>
         </is>
       </c>
     </row>
@@ -7374,18 +8213,129 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
+          <t>거래 가능일 245일 · 등록 권장 2,011 kW · 연간 감축 34,350 kWh</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>R1 용인 실측</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>7.1 선택요금 전환</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>높음</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>II → II</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>7.2 계약전력 조정</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>높음</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>계약 290 kW (실제 값)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>7.4 역률 개선 (92→97%)</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>124225.2129032239</v>
+      </c>
+      <c r="D39" t="n">
+        <v>124225.2129032239</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>높음</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>요금표와 약관만으로 확정</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>7.6 ESS</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>중간~낮음</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>최소 규격 미달 — 필요 출력 25.3 kW &lt; 상업용 최소 50 kW</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>7.3 경제성DR</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>중간</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
           <t>거래 가능일 244일 · 등록 권장 28 kW · 연간 감축 5,882 kWh</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
     <mergeCell ref="A22:A26"/>
     <mergeCell ref="A17:A21"/>
     <mergeCell ref="A12:A16"/>
     <mergeCell ref="A27:A31"/>
     <mergeCell ref="A2:A6"/>
     <mergeCell ref="A7:A11"/>
+    <mergeCell ref="A37:A41"/>
     <mergeCell ref="A32:A36"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7398,7 +8348,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D105"/>
+  <dimension ref="A1:D119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8884,7 +9834,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>R1 용인 실측</t>
+          <t>C7 계약 부족형</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -8916,7 +9866,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>0 → 21,832,794 → 23,715,557 → 24,660,959</t>
+          <t>0 → 78,883,247 → 157,766,493 → 315,532,987</t>
         </is>
       </c>
     </row>
@@ -8933,7 +9883,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>증분 1,371,755 → 49,380 → 0</t>
+          <t>증분 12,693,662 → 5,217,352 → 3,924,070</t>
         </is>
       </c>
     </row>
@@ -8950,7 +9900,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>132.0 → 120.0 → 120.0 → 120.0</t>
+          <t>5,293.0 → 5,204.0 → 5,198.0 → 5,186.0</t>
         </is>
       </c>
     </row>
@@ -8967,7 +9917,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>최대 편차 0.002%</t>
+          <t>최대 편차 0.017%</t>
         </is>
       </c>
     </row>
@@ -9001,7 +9951,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>기본요금 절감액 상한: 평탄형</t>
+          <t>기본요금 절감액 상한: 기준, 평탄형</t>
         </is>
       </c>
     </row>
@@ -9018,7 +9968,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>0 원 · II → II</t>
+          <t>34,923,556 원 · I → II</t>
         </is>
       </c>
     </row>
@@ -9035,7 +9985,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>124,225 원 (기본요금 12,422,521 의 1.00%)</t>
+          <t>4,528,046 원 (기본요금 452,804,556 의 1.00%)</t>
         </is>
       </c>
     </row>
@@ -9052,7 +10002,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>244 / 365일</t>
+          <t>245 / 359일</t>
         </is>
       </c>
     </row>
@@ -9069,7 +10019,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>viable=False · 목표 0 kW</t>
+          <t>viable=True · 목표 5,180 kW</t>
         </is>
       </c>
     </row>
@@ -9086,7 +10036,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>목표 0 kW · 절감액 —</t>
+          <t>목표 5,180 kW · 절감액 25,544,657 원</t>
         </is>
       </c>
     </row>
@@ -9103,7 +10053,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>어긋난 점 0개 / 0개</t>
+          <t>어긋난 점 0개 / 21개</t>
         </is>
       </c>
     </row>
@@ -9120,19 +10070,19 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>어긋난 점 0개 / 0개</t>
+          <t>어긋난 점 0개 / 21개</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>교차</t>
+          <t>R1 용인 실측</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>C1 오전 피크형 &gt; C2 오후 피크형 (요금적용전력 저감 폭)</t>
+          <t>PV 0 kWp 절감액이 정확히 0</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -9142,14 +10092,14 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>C1 95.0 kW vs C2 5.0 kW — C2 는 피크가 늦어 PV 가 깎은 뒤 저녁 슬롯이 새 최대가 된다</t>
+          <t>0.000000 원</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="B101" t="inlineStr">
         <is>
-          <t>C3 평탄형은 기본요금 절감이 거의 없다 (절감의 대부분이 전력량요금)</t>
+          <t>용량 증가 시 전력량요금 절감액 단조 증가</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -9159,14 +10109,14 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>기본요금 비중 C3 3.6% vs C1 10.2% (C3 저감 26.0 kW)</t>
+          <t>0 → 21,832,794 → 23,715,557 → 24,660,959</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="B102" t="inlineStr">
         <is>
-          <t>C5 겨울 피크형은 기본요금 절감이 매우 작다</t>
+          <t>기본요금 절감액 단조 증가 후 포화</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -9176,14 +10126,14 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>저감률 C5 0.29% vs C1 1.79% — 겨울 대상월의 피크가 07~09시·17~20시라 PV 가 닿지 않는다</t>
+          <t>증분 1,371,755 → 49,380 → 0</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="B103" t="inlineStr">
         <is>
-          <t>C6 야간 피크형: 요금적용전력 &lt; 관측 최대수요 (경부하 제외, 5.2 ①)</t>
+          <t>용량 증가 시 요금적용전력 단조 감소</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -9193,14 +10143,14 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>관측 10,920.6 kW vs 요금적용 3,604.0 kW (67.0% 낮다)</t>
+          <t>132.0 → 120.0 → 120.0 → 120.0</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="B104" t="inlineStr">
         <is>
-          <t>C6 야간 피크형: 하한이 요금적용전력을 붙들어 PV 가 한 칸도 못 내린다</t>
+          <t>감도 세 시나리오의 발전량이 ±1% 이내 (총량 보존)</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -9210,35 +10160,279 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>C6 저감 0.00 kW vs C1 95.00 kW — 경부하 최대라 대상 수요가 하한 3,603.8 kW 아래에 있다</t>
+          <t>최대 편차 0.002%</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="B105" t="inlineStr">
         <is>
+          <t>기준값이 범위 안에 있음</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>통과</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>벗어난 지표 0건</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>상한 시나리오 기록 (단조성은 요구하지 않는다)</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>통과</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>기본요금 절감액 상한: 평탄형</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>선택요금 전환 절감액 ≥ 0 (확정 계산)</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>통과</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>0 원 · II → II</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>역률 개선 절감액 = 기본요금의 1.0% (감액 상한)</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>통과</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>124,225 원 (기본요금 12,422,521 의 1.00%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>DR 거래 가능일이 전체 일수보다 적음 (토·일·공휴일 제외)</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>통과</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>244 / 365일</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>ESS 성립하지 않으면 목표가 0 (없는 목표를 내지 않는다)</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>통과</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>viable=False · 목표 0 kW</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>ESS 목표를 냈으면 절감액 &gt; 0</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>통과</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>목표 0 kW · 절감액 —</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>ESS 목표 달성이면 실제 요금적용전력이 목표 이하</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>통과</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>어긋난 점 0개 / 0개</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>ESS 절감액이 0 이하인 점에는 회수기간이 없다</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>통과</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>어긋난 점 0개 / 0개</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>교차</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>C1 오전 피크형 &gt; C2 오후 피크형 (요금적용전력 저감 폭)</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>통과</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>C1 95.0 kW vs C2 5.0 kW — C2 는 피크가 늦어 PV 가 깎은 뒤 저녁 슬롯이 새 최대가 된다</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>C3 평탄형은 기본요금 절감이 거의 없다 (절감의 대부분이 전력량요금)</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>통과</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>기본요금 비중 C3 3.6% vs C1 10.2% (C3 저감 26.0 kW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>C5 겨울 피크형은 기본요금 절감이 매우 작다</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>통과</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>저감률 C5 0.29% vs C1 1.79% — 겨울 대상월의 피크가 07~09시·17~20시라 PV 가 닿지 않는다</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>C6 야간 피크형: 요금적용전력 &lt; 관측 최대수요 (경부하 제외, 5.2 ①)</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>통과</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>관측 10,920.6 kW vs 요금적용 3,604.0 kW (67.0% 낮다)</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>C6 야간 피크형: 하한이 요금적용전력을 붙들어 PV 가 한 칸도 못 내린다</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>통과</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>C6 저감 0.00 kW vs C1 95.00 kW — 경부하 최대라 대상 수요가 하한 3,603.8 kW 아래에 있다</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="B119" t="inlineStr">
+        <is>
           <t>C4 산업용(을) 주말 할인이 PV 최성기와 겹쳐 전력량요금 절감 비율이 낮다</t>
         </is>
       </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>통과</t>
-        </is>
-      </c>
-      <c r="D105" t="inlineStr">
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>통과</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
         <is>
           <t>C4 4.95% vs C1 5.44% (봄·가을 토·일·공휴일 11~14시 할인 구간의 단가가 이미 낮다)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A30:A43"/>
     <mergeCell ref="A44:A57"/>
     <mergeCell ref="A16:A29"/>
+    <mergeCell ref="A114:A119"/>
+    <mergeCell ref="A100:A113"/>
     <mergeCell ref="A72:A85"/>
     <mergeCell ref="A86:A99"/>
-    <mergeCell ref="A100:A105"/>
     <mergeCell ref="A2:A15"/>
     <mergeCell ref="A58:A71"/>
   </mergeCells>
@@ -9252,7 +10446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9275,7 +10469,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>23.6 초</t>
+          <t>22.8 초</t>
         </is>
       </c>
     </row>
@@ -9287,7 +10481,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>23.0 초</t>
+          <t>22.9 초</t>
         </is>
       </c>
     </row>
@@ -9311,7 +10505,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>24.1 초</t>
+          <t>23.5 초</t>
         </is>
       </c>
     </row>
@@ -9323,7 +10517,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>25.6 초</t>
+          <t>25.5 초</t>
         </is>
       </c>
     </row>
@@ -9335,55 +10529,67 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>19.8 초</t>
+          <t>19.7 초</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>R1 용인 실측 소요</t>
+          <t>C7 계약 부족형 소요</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>32.9 초</t>
+          <t>24.1 초</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>전체 소요</t>
+          <t>R1 용인 실측 소요</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>170.2 초</t>
+          <t>33.2 초</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>기상 취득 호출</t>
+          <t>전체 소요</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0 회</t>
+          <t>192.9 초</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>기상 취득 호출</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0 회</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>기상 캐시 적중</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>7/7 (합성 여섯은 좌표·기간이 같아 첫 건만 취득한다. 실측은 따로 선다)</t>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>8/8 (C1~C7 은 좌표·기간이 같아 첫 건만 취득한다. 실측은 따로 선다)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
S129 3절: 마감 - 케이스 118/118 · pytest 1,667 · 미해결 58 -> 59
케이스 118/118 · 도구 193.6초 / 벽시계 201초 · 기상 취득 0회 · 깨끗한 판 ·
회귀값 여덟 불변.

감사 956·806·959·807 -> 957·807·961·808. 화면 명세에 역률 열이 넷 다 +1,
부가금 열이 부가금 서는 종별 둘에 +1 이다. screen_budget 모든 자리 한도 안.
scan_ctrl 제어문자 0 · 탭 0. ruff check 통과. 맨 mypy 고친 세 파일 통과.
ruff format 은 test_excess.py 가 어긋나는데 HEAD 에서도 같아 이 판이 낸 것이
아니다 (2-28).

pytest 1,666 -> 1,667 (2번 PC 갈래 넷 합 12분 23초 · 넷 다 깨끗한 판).
갈래 합 1,036 + 232 + 58 + 341 = 1,667 이라 수집과 같다.

2-32 를 값으로 판정했다 - 이름의 절반이 틀렸다. 역률요금은 이미 담기고 안
담기는 것은 부가금 하나뿐이다. 109세션이 「사람이 정한다」 로 열어 둔 자리라
판정까지만 했다.

미해결 58 -> 59 (늘어난 것 2-51 「기본요금」 이 산출물마다 다른 몫을 센다 ·
줄어든 것 없음).

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vr2pjktJG7fxenaYX4Ph5J
</commit_message>
<xml_diff>
--- a/output/casestudy_20260906.xlsx
+++ b/output/casestudy_20260906.xlsx
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>22.78387420019135</v>
+        <v>22.7837538998574</v>
       </c>
     </row>
     <row r="3">
@@ -596,7 +596,7 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>22.94120769994333</v>
+        <v>22.98959789983928</v>
       </c>
     </row>
     <row r="4">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>15.08017049985938</v>
+        <v>15.19798669987358</v>
       </c>
     </row>
     <row r="5">
@@ -700,7 +700,7 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>23.54686559992842</v>
+        <v>23.90659380005673</v>
       </c>
     </row>
     <row r="6">
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>25.51196929998696</v>
+        <v>25.65873919986188</v>
       </c>
     </row>
     <row r="7">
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>19.7029236999806</v>
+        <v>19.85932990000583</v>
       </c>
     </row>
     <row r="8">
@@ -856,7 +856,7 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>24.07502040010877</v>
+        <v>24.1428493000567</v>
       </c>
     </row>
     <row r="9">
@@ -908,7 +908,7 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>33.19355620001443</v>
+        <v>32.9609304999467</v>
       </c>
     </row>
   </sheetData>
@@ -10481,7 +10481,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>22.9 초</t>
+          <t>23.0 초</t>
         </is>
       </c>
     </row>
@@ -10493,7 +10493,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.1 초</t>
+          <t>15.2 초</t>
         </is>
       </c>
     </row>
@@ -10505,7 +10505,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>23.5 초</t>
+          <t>23.9 초</t>
         </is>
       </c>
     </row>
@@ -10517,7 +10517,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>25.5 초</t>
+          <t>25.7 초</t>
         </is>
       </c>
     </row>
@@ -10529,7 +10529,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>19.7 초</t>
+          <t>19.9 초</t>
         </is>
       </c>
     </row>
@@ -10553,7 +10553,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>33.2 초</t>
+          <t>33.0 초</t>
         </is>
       </c>
     </row>
@@ -10565,7 +10565,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>192.9 초</t>
+          <t>193.6 초</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
S134 4절: 마감 - 갈래 넷 1,679건 · 미해결 64 -> 64 · 살아 있는 못 1 -> 1
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KtMDWiB2gkNwrcE4nNgoA6
</commit_message>
<xml_diff>
--- a/output/casestudy_20260906.xlsx
+++ b/output/casestudy_20260906.xlsx
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>23.33048870018683</v>
+        <v>23.01522890012711</v>
       </c>
     </row>
     <row r="3">
@@ -596,7 +596,7 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>23.35353829991072</v>
+        <v>23.17185600008816</v>
       </c>
     </row>
     <row r="4">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>15.47251340001822</v>
+        <v>15.28280719998293</v>
       </c>
     </row>
     <row r="5">
@@ -700,7 +700,7 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>24.17340570013039</v>
+        <v>24.0123493000865</v>
       </c>
     </row>
     <row r="6">
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>26.04440349992365</v>
+        <v>25.8732350000646</v>
       </c>
     </row>
     <row r="7">
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>20.13997430005111</v>
+        <v>20.01492530014366</v>
       </c>
     </row>
     <row r="8">
@@ -856,7 +856,7 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>24.58694879990071</v>
+        <v>24.40131260012276</v>
       </c>
     </row>
     <row r="9">
@@ -908,7 +908,7 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>33.69574179989286</v>
+        <v>33.68226990010589</v>
       </c>
     </row>
   </sheetData>
@@ -7972,7 +7972,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>목표 5,970 kW (기준 6,175.0 → 실제 5,970.0) · 250 kW / 200 kWh · 회수 56.1년</t>
+          <t>목표 5,970 kW (기준 6,175.0 → 실제 5,970.0) · 250 kW / 200 kWh · 회수 &gt;50년</t>
         </is>
       </c>
     </row>
@@ -10469,7 +10469,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>23.3 초</t>
+          <t>23.0 초</t>
         </is>
       </c>
     </row>
@@ -10481,7 +10481,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>23.4 초</t>
+          <t>23.2 초</t>
         </is>
       </c>
     </row>
@@ -10493,7 +10493,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.5 초</t>
+          <t>15.3 초</t>
         </is>
       </c>
     </row>
@@ -10505,7 +10505,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>24.2 초</t>
+          <t>24.0 초</t>
         </is>
       </c>
     </row>
@@ -10517,7 +10517,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>26.0 초</t>
+          <t>25.9 초</t>
         </is>
       </c>
     </row>
@@ -10529,7 +10529,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>20.1 초</t>
+          <t>20.0 초</t>
         </is>
       </c>
     </row>
@@ -10541,7 +10541,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>24.6 초</t>
+          <t>24.4 초</t>
         </is>
       </c>
     </row>
@@ -10565,7 +10565,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>196.9 초</t>
+          <t>195.5 초</t>
         </is>
       </c>
     </row>

</xml_diff>